<commit_message>
Bridge MMTO Cost Working
</commit_message>
<xml_diff>
--- a/data/BenchmarkDatabaseCost.xlsx
+++ b/data/BenchmarkDatabaseCost.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Krishnan Suresh\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00E51978-3266-4028-A38B-9D7040274C35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{520BA14F-22C8-4326-93A7-3E7C1D6F5735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
   <si>
     <t>Material</t>
   </si>
@@ -76,9 +76,6 @@
   </si>
   <si>
     <t>Cost</t>
-  </si>
-  <si>
-    <t>D</t>
   </si>
 </sst>
 </file>
@@ -108,18 +105,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="4">
@@ -175,7 +166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -208,18 +199,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="11" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -536,24 +515,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M5"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M4"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
-    <col min="2" max="2" width="5.85546875" customWidth="1"/>
-    <col min="3" max="3" width="8.42578125" customWidth="1"/>
-    <col min="4" max="4" width="24.140625" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="18.28515625" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" customWidth="1"/>
-    <col min="7" max="7" width="10.85546875" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="24.85546875" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="25.5703125" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="21.42578125" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="21.42578125" customWidth="1"/>
-    <col min="12" max="12" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="2" width="5.88671875" customWidth="1"/>
+    <col min="3" max="3" width="8.44140625" customWidth="1"/>
+    <col min="4" max="4" width="24.109375" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="18.33203125" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" customWidth="1"/>
+    <col min="7" max="7" width="10.88671875" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="24.88671875" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="25.5546875" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="21.44140625" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="21.44140625" customWidth="1"/>
+    <col min="12" max="12" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -594,7 +573,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>13</v>
       </c>
@@ -635,7 +614,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>14</v>
       </c>
@@ -676,7 +655,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>15</v>
       </c>
@@ -714,47 +693,6 @@
         <v>0.87</v>
       </c>
       <c r="M4" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="13">
-        <v>0</v>
-      </c>
-      <c r="D5" s="13">
-        <v>1240</v>
-      </c>
-      <c r="E5" s="13">
-        <v>1035</v>
-      </c>
-      <c r="F5" s="14">
-        <v>1E-3</v>
-      </c>
-      <c r="G5" s="13">
-        <v>7</v>
-      </c>
-      <c r="H5" s="13">
-        <v>1400</v>
-      </c>
-      <c r="I5" s="13">
-        <v>980</v>
-      </c>
-      <c r="J5" s="13">
-        <v>12</v>
-      </c>
-      <c r="K5" s="14">
-        <v>1E-10</v>
-      </c>
-      <c r="L5" s="15">
-        <v>0.87</v>
-      </c>
-      <c r="M5" s="15">
         <v>1</v>
       </c>
     </row>

</xml_diff>